<commit_message>
@ feat(FL1-03): bộ câu hỏi theo khung CT + điểm/thời gian/ảnh + template
Question form đủ trường (curriculumId/courseId/points/timeLimitSec/imageUrl +
choice.imageUrl/explanation); lọc list+picker theo khung CT; import Excel thêm
cột courseSlug/curriculumVersion/points/timeLimitSec + template mẫu. Helper
buildQuestionWhere dùng chung. Test 18/18.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/public/templates/mau-ngan-hang-cau-hoi.xlsx
+++ b/public/templates/mau-ngan-hang-cau-hoi.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:U4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,39 +416,51 @@
         <v>tags</v>
       </c>
       <c r="F1" t="str">
+        <v>courseSlug</v>
+      </c>
+      <c r="G1" t="str">
+        <v>curriculumVersion</v>
+      </c>
+      <c r="H1" t="str">
+        <v>points</v>
+      </c>
+      <c r="I1" t="str">
+        <v>timeLimitSec</v>
+      </c>
+      <c r="J1" t="str">
         <v>correctAnswer</v>
       </c>
-      <c r="G1" t="str">
+      <c r="K1" t="str">
         <v>choice1</v>
       </c>
-      <c r="H1" t="str">
+      <c r="L1" t="str">
         <v>choice1_correct</v>
       </c>
-      <c r="I1" t="str">
+      <c r="M1" t="str">
         <v>choice2</v>
       </c>
-      <c r="J1" t="str">
+      <c r="N1" t="str">
         <v>choice2_correct</v>
       </c>
-      <c r="K1" t="str">
+      <c r="O1" t="str">
         <v>choice3</v>
       </c>
-      <c r="L1" t="str">
+      <c r="P1" t="str">
         <v>choice3_correct</v>
       </c>
-      <c r="M1" t="str">
+      <c r="Q1" t="str">
         <v>choice4</v>
       </c>
-      <c r="N1" t="str">
+      <c r="R1" t="str">
         <v>choice4_correct</v>
       </c>
-      <c r="O1" t="str">
+      <c r="S1" t="str">
         <v>explanation</v>
       </c>
-      <c r="P1" t="str">
+      <c r="T1" t="str">
         <v>isPublic</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="U1" t="str">
         <v>notes</v>
       </c>
     </row>
@@ -469,39 +481,51 @@
         <v>robosim, movement, basic</v>
       </c>
       <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
+        <v>lap-trinh-robot</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>60</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
         <v>Tiến</v>
       </c>
-      <c r="H2" t="str">
+      <c r="L2" t="str">
         <v>TRUE</v>
       </c>
-      <c r="I2" t="str">
+      <c r="M2" t="str">
         <v>Lùi</v>
-      </c>
-      <c r="J2" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Bay</v>
-      </c>
-      <c r="L2" t="str">
-        <v>FALSE</v>
-      </c>
-      <c r="M2" t="str">
-        <v>Quay trái/phải</v>
       </c>
       <c r="N2" t="str">
         <v>TRUE</v>
       </c>
       <c r="O2" t="str">
+        <v>Bay</v>
+      </c>
+      <c r="P2" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Quay trái/phải</v>
+      </c>
+      <c r="R2" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="S2" t="str">
         <v>Robot Robosim chỉ di chuyển trên mặt phẳng, không thể bay</v>
       </c>
-      <c r="P2" t="str">
+      <c r="T2" t="str">
         <v>TRUE</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="U2" t="str">
         <v/>
       </c>
     </row>
@@ -522,39 +546,51 @@
         <v>loop, programming</v>
       </c>
       <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
+        <v>lap-trinh-robot</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>45</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
         <v>Đúng</v>
       </c>
-      <c r="H3" t="str">
+      <c r="L3" t="str">
         <v>FALSE</v>
       </c>
-      <c r="I3" t="str">
+      <c r="M3" t="str">
         <v>Sai</v>
       </c>
-      <c r="J3" t="str">
+      <c r="N3" t="str">
         <v>TRUE</v>
       </c>
-      <c r="K3" t="str">
-        <v/>
-      </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
-        <v/>
-      </c>
-      <c r="N3" t="str">
-        <v/>
-      </c>
       <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
         <v>Vòng for có biến đếm và giới hạn rõ ràng, khác while(true)</v>
       </c>
-      <c r="P3" t="str">
+      <c r="T3" t="str">
         <v>TRUE</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="U3" t="str">
         <v/>
       </c>
     </row>
@@ -575,20 +611,20 @@
         <v>python, output, function</v>
       </c>
       <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
         <v>print</v>
       </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
       <c r="K4" t="str">
         <v/>
       </c>
@@ -602,18 +638,30 @@
         <v/>
       </c>
       <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
         <v>print() là built-in function của Python</v>
       </c>
-      <c r="P4" t="str">
+      <c r="T4" t="str">
         <v>TRUE</v>
       </c>
-      <c r="Q4" t="str">
+      <c r="U4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>